<commit_message>
feat(scripts): broaden constant naming, opt-in backups, .bak-safe discovery
</commit_message>
<xml_diff>
--- a/Excel/11_Wastewater_WIP_v02.xlsx
+++ b/Excel/11_Wastewater_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9297710D-CBA7-4A43-A6C8-494BE58D6622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B807BA1-44C2-404C-B1E2-E854BDD9954D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15345" firstSheet="7" activeTab="7" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" firstSheet="7" activeTab="7" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -262,6 +262,11 @@
     <definedName name="Step3">#REF!</definedName>
     <definedName name="VEERG_11_1_1_1__1_MethaneEmissionsFromWastewaterTreatment_Result_Method1">'11.1.1-2 Wastewater CH4'!$E$30</definedName>
     <definedName name="VEERG_11_1_3_1__1_NitrousOxideEmissionsFromFlaredBiogas_Result_Method1">'11.1.3-4 Wastewater N2O'!$E$17</definedName>
+    <definedName name="Waste_EnergyContentFactorSludgeBiogasFlared_Data">'Constants - Wastewater'!$E$41</definedName>
+    <definedName name="Waste_MethaneEmissionFactorSludge_Data">'Constants - Wastewater'!$E$36</definedName>
+    <definedName name="Waste_MethaneEmissionFactorSludgeBiogasFlared_Data">'Constants - Wastewater'!$E$46</definedName>
+    <definedName name="Waste_MethaneEmissionFactorWastewater_Data">'Constants - Wastewater'!$E$31</definedName>
+    <definedName name="Waste_NitrousOxideEmissionFactorSludgeBiogasFlared_Data">'Constants - Wastewater'!$E$51</definedName>
     <definedName name="Wastewater_Methane_Equations.VEERG_11_1_1_1__1_MethaneEmissionsFromWastewaterTreatment">_xlfn.LAMBDA(_xlpm.W_t,_xlpm.COD_in,_xlpm.F_sludge,_xlpm.COD_out,_xlpm.CF_ww_t,_xlpm.EF_ww,_xlpm.F_removed,_xlpm.CF_sludge_t,_xlpm.EF_sludge,_xlpm.Q_cap,_xlpm.Q_flared,_xlpm.Q_out,_xlpm.EC_flared,_xlpm.EF_flaredCH4, (1 / 1000) * ((_xlpm.W_t * (_xlpm.COD_in * (1 - _xlpm.F_sludge) - _xlpm.COD_out) * _xlpm.CF_ww_t * _xlpm.EF_ww) + (_xlpm.W_t * (_xlpm.COD_in * (_xlpm.F_sludge - _xlpm.F_removed)) * _xlpm.CF_sludge_t * _xlpm.EF_sludge) - (6.784 * 10 ^ -4 * (_xlpm.Q_cap + _xlpm.Q_flared + _xlpm.Q_out)) + (_xlpm.Q_flared * (_xlpm.EC_flared * _xlpm.EF_flaredCH4))))</definedName>
     <definedName name="Wastewater_Methane_Equations.VEERG_11_1_1_1__1_MethaneEmissionsFromWastewaterTreatment_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(15, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"W_t","quantity of wastewater treated at facility type t","m3","Input";"COD_in","average inlet Chemical Oxygen Demand concentration of wastewater","kg COD/m3","Input";"F_sludge","fraction of COD removed from wastewater as sludge","fraction","Input";"COD_out","average outlet COD concentration of wastewater","kg COD/m3","Input";"CF_ww_t","methane correction factor for facility type t used to treat wastewater","fraction","Constant";"EF_ww","methane emission factor for wastewater","kg CH4/kg COD","Constant";"F_removed","fraction of COD removed from the wastewater treatment facility and transferred elsewhere","fraction","Input";"CF_sludge_t","methane correction factor for facility type t used to treat sludge","fraction","Constant";"EF_sludge","methane emission factor for sludge","kg CH4/kg COD","Constant";"Q_cap","quantity of methane in sludge biogas captured for combustion","m3 CH4","Input";"Q_flared","quantity of methane in sludge biogas flared by the treatment facility","m3 CH4","Input";"Q_out","quantity of methane in sludge biogas transferred out of the treatment facility","m3 CH4","Input";"EC_flared","energy content factor of methane in sludge biogas flared","GJ/m3","Constant";"EF_flaredCH4","methane emission factor for sludge biogas flared","kg CH4/GJ","Constant";"t","treatment facility type","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Wastewater_Methane_Equations.VEERG_11_1_1_1__1_MethaneEmissionsFromWastewaterTreatment_LatexEquation">_xlfn.LAMBDA(_xlfn._LONGTEXT("E_{CH4}=\frac{1}{1000}\times\left{\left{W_t\times\left[COD_{in}\times(1-F_{sludge})-COD_{out}\right]\times CF_{ww,t}\times EF_{ww}\right}+\left{W_t\times\left[COD_{in}\times(F_{sludge}-F_{removed})\right]\times CF_{sludge,t}\times EF_{sludge}\right}-\left","{6.784\times 10^{-4}\times \left[ Q_{cap}+Q_{flared}+Q_{out}\right]\right}+\left{Q_{flared}\times \left[ EC_{flared}\times EF_{flared,CH4}\right]\right}\right}"))</definedName>
@@ -7722,7 +7727,7 @@
     </row>
     <row r="57" spans="4:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D57" s="1">
-        <f>F8*(F14*(1-F15)-F17)</f>
+        <f>X_Cell_Wastewater_QuantityInM3*(X_Cell_Wastewater_InletCOD*(1-X_Cell_Wastewater_FractionCODRemovedAsSludge)-X_Cell_Wastewater_OutletCOD)</f>
         <v>350</v>
       </c>
     </row>
@@ -8050,8 +8055,8 @@
       <c r="D8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="10" t="str" cm="1">
-        <f t="array" aca="1" ref="E8" ca="1">Common_InputFunctions.Utility_DisplayFunctionName(E30)</f>
+      <c r="E8" s="10" t="str">
+        <f ca="1">Common_InputFunctions.Utility_DisplayFunctionName(VEERG_11_1_1_1__1_MethaneEmissionsFromWastewaterTreatment_Result_Method1)</f>
         <v>=Wastewater_Methane_Equations.VEERG_11_1_1_1__1_MethaneEmissionsFromWastewaterTreatment</v>
       </c>
     </row>
@@ -8222,7 +8227,7 @@
         <v>Constant</v>
       </c>
       <c r="J19" s="44">
-        <f>'Constants - Wastewater'!$E$31</f>
+        <f>Waste_MethaneEmissionFactorWastewater_Data</f>
         <v>0.25</v>
       </c>
     </row>
@@ -8282,7 +8287,7 @@
         <v>Constant</v>
       </c>
       <c r="J22" s="44">
-        <f>'Constants - Wastewater'!$E$36</f>
+        <f>Waste_MethaneEmissionFactorSludge_Data</f>
         <v>0.25</v>
       </c>
     </row>
@@ -8362,7 +8367,7 @@
         <v>Constant</v>
       </c>
       <c r="J26" s="44">
-        <f>'Constants - Wastewater'!$E$41</f>
+        <f>Waste_EnergyContentFactorSludgeBiogasFlared_Data</f>
         <v>3.7699999999999997E-2</v>
       </c>
     </row>
@@ -8382,7 +8387,7 @@
         <v>Constant</v>
       </c>
       <c r="J27" s="44">
-        <f>'Constants - Wastewater'!$E$46</f>
+        <f>Waste_MethaneEmissionFactorSludgeBiogasFlared_Data</f>
         <v>0.22889999999999999</v>
       </c>
     </row>
@@ -8431,7 +8436,7 @@
       </c>
       <c r="F32" s="68"/>
       <c r="G32" s="26">
-        <f>E30</f>
+        <f>VEERG_11_1_1_1__1_MethaneEmissionsFromWastewaterTreatment_Result_Method1</f>
         <v>4.7159433000000001E-2</v>
       </c>
     </row>
@@ -8779,8 +8784,8 @@
       <c r="D7" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="10" t="str" cm="1">
-        <f t="array" aca="1" ref="E7" ca="1">Common_InputFunctions.Utility_DisplayFunctionName(E17)</f>
+      <c r="E7" s="10" t="str">
+        <f ca="1">Common_InputFunctions.Utility_DisplayFunctionName(VEERG_11_1_3_1__1_NitrousOxideEmissionsFromFlaredBiogas_Result_Method1)</f>
         <v>=Wastewater_N2O_Equations.VEERG_11_1_3_1__1_NitrousOxideEmissionsFromFlaredBiogas</v>
       </c>
     </row>
@@ -8862,7 +8867,7 @@
         <v>Constant</v>
       </c>
       <c r="I14" s="44">
-        <f>'Constants - Wastewater'!E41</f>
+        <f>Waste_EnergyContentFactorSludgeBiogasFlared_Data</f>
         <v>3.7699999999999997E-2</v>
       </c>
     </row>
@@ -8881,7 +8886,7 @@
         <v>Constant</v>
       </c>
       <c r="I15" s="44">
-        <f>'Constants - Wastewater'!E51</f>
+        <f>Waste_NitrousOxideEmissionFactorSludgeBiogasFlared_Data</f>
         <v>1.132E-4</v>
       </c>
     </row>
@@ -8922,7 +8927,7 @@
       </c>
       <c r="F19" s="68"/>
       <c r="G19" s="26">
-        <f>E17</f>
+        <f>VEERG_11_1_3_1__1_NitrousOxideEmissionsFromFlaredBiogas_Result_Method1</f>
         <v>4.26764E-7</v>
       </c>
     </row>

</xml_diff>